<commit_message>
Cleaned up board shapes so that PCB will ship with cutouts for the DIN rail adapter clips
</commit_message>
<xml_diff>
--- a/ESP32_S3_DevKitC_1_1v1/ESP_32_S3_DevkitC_v1_1_Breakout/BOM_2026_03_22.xlsx
+++ b/ESP32_S3_DevKitC_1_1v1/ESP_32_S3_DevkitC_v1_1_Breakout/BOM_2026_03_22.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agmot\Documents\gitRepos\Public_PCBs\ESP32_S3_DevKitC_1_1v1\ESP_32_S3_DevkitC_v1_1_Breakout\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2f3a43259e44ff0e/Documents/KiCAD_Projects/ESP_32_S3_DevkitC_v1_1_Breakout/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06C0B341-61C6-414C-9CDE-40058CFFA341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{B574D405-4389-49CA-865A-0D7A9CECF5F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{984C495F-4559-4ED8-9098-E61D1BA0728E}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-11100" windowWidth="16440" windowHeight="28320" xr2:uid="{ADA09AAB-AFE2-4520-BD01-3AF7A48FFB9E}"/>
+    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="9960" xr2:uid="{ADA09AAB-AFE2-4520-BD01-3AF7A48FFB9E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="21">
   <si>
     <t>Item</t>
   </si>
@@ -50,6 +50,9 @@
     <t>Link</t>
   </si>
   <si>
+    <t>CONN HDR 22POS 0.1 GOLD PCB</t>
+  </si>
+  <si>
     <t>Line Price</t>
   </si>
   <si>
@@ -65,6 +68,9 @@
     <t>https://www.digikey.com/en/products/detail/phoenix-contact/1990203/950942</t>
   </si>
   <si>
+    <t>PPPC112LFBN_RC</t>
+  </si>
+  <si>
     <t>DINRAIL ADAPTER UNIVERSAL</t>
   </si>
   <si>
@@ -93,33 +99,6 @@
   </si>
   <si>
     <t>https://www.digikey.com/en/products/detail/samtec-inc/SSW-122-01-F-D/7882389</t>
-  </si>
-  <si>
-    <t>CONN HDR 44 POS 2 ROW 0.1 GOLD PCB</t>
-  </si>
-  <si>
-    <t>CONN HEADER SMD R/A 4POS 1MM</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/jst-sales-america-inc/SM04B-SRSS-TB/926710</t>
-  </si>
-  <si>
-    <t>SM04B-SRSS-TB</t>
-  </si>
-  <si>
-    <t>SSW-122-01-F-D</t>
-  </si>
-  <si>
-    <t>M3x8mm Machine Screw, SS BtnHd, Hex</t>
-  </si>
-  <si>
-    <t>https://www.mcmaster.com/products/screws/rounded-head-screws-2~/stainless-steel-button-head-hex-drive-screws~~/</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Pack of 100</t>
   </si>
 </sst>
 </file>
@@ -151,7 +130,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -176,12 +155,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -196,14 +169,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -539,18 +511,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D3C3D0-0B48-458B-B6CE-0B6172BCB0EE}">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.77734375" customWidth="1"/>
     <col min="7" max="7" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -562,246 +533,153 @@
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="C2">
         <v>4.2300000000000004</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E2">
         <f>C2*D2</f>
-        <v>8.4600000000000009</v>
+        <v>29.610000000000003</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" s="3">
         <v>4.3099999999999996</v>
       </c>
       <c r="D3" s="3">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E3" s="3">
         <f>C3*D3</f>
-        <v>8.6199999999999992</v>
+        <v>30.169999999999998</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G3" s="3">
         <v>1990203</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C4">
         <v>1.24</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E4">
         <f>C4*D4</f>
-        <v>2.48</v>
+        <v>8.68</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5">
-        <v>0.5</v>
-      </c>
-      <c r="D5">
-        <v>2</v>
-      </c>
-      <c r="E5">
-        <f>C5*D5</f>
-        <v>1</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6">
-        <v>8.8000000000000007</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <f>C6*D6</f>
-        <v>8.8000000000000007</v>
-      </c>
-      <c r="F6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G6" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="L6" s="6" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" t="s">
-        <v>11</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>